<commit_message>
Update inventory for new - 1782560254707
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Sno</t>
   </si>
@@ -30,6 +30,24 @@
   </si>
   <si>
     <t>Location</t>
+  </si>
+  <si>
+    <t>7774005800239041</t>
+  </si>
+  <si>
+    <t>4902470171036</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>20-40-60</t>
   </si>
 </sst>
 </file>
@@ -93,7 +111,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
@@ -124,6 +142,26 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s" s="1">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s" s="1">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Update inventory for new - 1782560398363
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Sno</t>
   </si>
@@ -30,24 +30,6 @@
   </si>
   <si>
     <t>Location</t>
-  </si>
-  <si>
-    <t>7774005800239041</t>
-  </si>
-  <si>
-    <t>4902470171036</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>20-40-60</t>
   </si>
 </sst>
 </file>
@@ -111,7 +93,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
@@ -142,26 +124,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s" s="1">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s" s="1">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s" s="1">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s" s="1">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s" s="1">
-        <v>11</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Update inventory for new - 1785241455678
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -126,6 +126,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t>899681002157</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
+        <is>
+          <t>1-2-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785242737463
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,6 +158,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>703878001031</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>3-3-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785242828475
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,38 +158,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr" s="2">
-        <is>
-          <t>703878001031</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="2">
-        <is>
-          <t>3-3-3</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785242942412
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,6 +158,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>703878001031</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>3-3-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785243021784
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,38 +158,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr" s="2">
-        <is>
-          <t>703878001031</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="2">
-        <is>
-          <t>3-3-3</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785243383468
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,6 +158,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>6281006424340</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>1-1-1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785243505651
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,38 +158,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr" s="2">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr" s="2">
-        <is>
-          <t>6281006424340</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr" s="2">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="2">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr" s="2">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="2">
-        <is>
-          <t>1-1-1</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785250195582
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -158,6 +158,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>8809782555508</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>11-11-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785252094253
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -190,6 +190,38 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t>50219056</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t>6-6-5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785253028942
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -222,6 +222,38 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t>6924526310020</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t>6-1-1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for new - 1785253365520
</commit_message>
<xml_diff>
--- a/stores/new.xlsx
+++ b/stores/new.xlsx
@@ -254,6 +254,38 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t>8886467080074</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t>7-7-7</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>